<commit_message>
repgrid sheet: poster columns named for the Drive folder entries (Grp 01..11)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etc/repgrid-sheet.xlsx
+++ b/etc/repgrid-sheet.xlsx
@@ -438,17 +438,17 @@
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="5.5" customWidth="1" min="3" max="3"/>
-    <col width="5.5" customWidth="1" min="4" max="4"/>
-    <col width="5.5" customWidth="1" min="5" max="5"/>
-    <col width="5.5" customWidth="1" min="6" max="6"/>
-    <col width="5.5" customWidth="1" min="7" max="7"/>
-    <col width="5.5" customWidth="1" min="8" max="8"/>
-    <col width="5.5" customWidth="1" min="9" max="9"/>
-    <col width="5.5" customWidth="1" min="10" max="10"/>
-    <col width="5.5" customWidth="1" min="11" max="11"/>
-    <col width="5.5" customWidth="1" min="12" max="12"/>
-    <col width="5.5" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="13" max="13"/>
     <col width="34" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -465,57 +465,57 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>poster 1  ·  g1–g2</t>
+          <t>Grp 01  ·  g1-g2</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>poster 2  ·  g1–g4</t>
+          <t>Grp 02  ·  g1-g4</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>poster 3  ·  g1–g6</t>
+          <t>Grp 03  ·  g1-g6</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>poster 4  ·  g3–g8</t>
+          <t>Grp 04  ·  g3-g8</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>poster 5  ·  g5–g10</t>
+          <t>Grp 05  ·  g5-g10</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>poster 6  ·  g7–g12</t>
+          <t>Grp 06  ·  g7-g12</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>poster 7  ·  g9–g14</t>
+          <t>Grp 07  ·  g9-g14</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>poster 8  ·  g11–g16</t>
+          <t>Grp 08  ·  g11-g16</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>poster 9  ·  g13–g17</t>
+          <t>Grp 09  ·  g13-g17</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>poster 10  ·  g15–g17</t>
+          <t>Grp 10  ·  g15-g17</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
         <is>
-          <t>poster 11  ·  g17–g17</t>
+          <t>Grp 11  ·  g17-g17</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
repgrid sheet: real project names in row 1 (WolfBite .. Howl2Go), from the poster PDFs
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etc/repgrid-sheet.xlsx
+++ b/etc/repgrid-sheet.xlsx
@@ -438,21 +438,21 @@
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
     <col width="34" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="90" customHeight="1">
+    <row r="1" ht="130" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>group</t>
@@ -465,57 +465,57 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Grp 01  ·  g1-g2</t>
+          <t>WolfBite  ·  g1-g2</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Grp 02  ·  g1-g4</t>
+          <t>Movie Munchers  ·  g1-g4</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Grp 03  ·  g1-g6</t>
+          <t>Weeklies  ·  g1-g6</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Grp 04  ·  g3-g8</t>
+          <t>Howl2Go (G4)  ·  g3-g8</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Grp 05  ·  g5-g10</t>
+          <t>Food Seer  ·  g5-g10</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Grp 06  ·  g7-g12</t>
+          <t>FoodPool  ·  g7-g12</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>Grp 07  ·  g9-g14</t>
+          <t>Hungry Wolf  ·  g9-g14</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>Grp 08  ·  g11-g16</t>
+          <t>TiffinTrails  ·  g11-g16</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>Grp 09  ·  g13-g17</t>
+          <t>MealPlan AI  ·  g13-g17</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>Grp 10  ·  g15-g17</t>
+          <t>MealSlot  ·  g15-g17</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
         <is>
-          <t>Grp 11  ·  g17-g17</t>
+          <t>Howl2Go (G11)  ·  g17-g17</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
repgrid sheet: headers carry project name + Drive file name + reviewer groups
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etc/repgrid-sheet.xlsx
+++ b/etc/repgrid-sheet.xlsx
@@ -452,7 +452,7 @@
     <col width="34" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="130" customHeight="1">
+    <row r="1" ht="170" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>group</t>
@@ -465,57 +465,57 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>WolfBite  ·  g1-g2</t>
+          <t>WolfBite · Group_1 · g1-g2</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Movie Munchers  ·  g1-g4</t>
+          <t>Movie Munchers · Group_2 · g1-g4</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Weeklies  ·  g1-g6</t>
+          <t>Weeklies · Group_3_Project_3 · g1-g6</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Howl2Go (G4)  ·  g3-g8</t>
+          <t>Howl2Go · Group_4 · g3-g8</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Food Seer  ·  g5-g10</t>
+          <t>Food Seer · Group_5 · g5-g10</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>FoodPool  ·  g7-g12</t>
+          <t>FoodPool · Group_6 · g7-g12</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>Hungry Wolf  ·  g9-g14</t>
+          <t>Hungry Wolf · Group_07 · g9-g14</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>TiffinTrails  ·  g11-g16</t>
+          <t>TiffinTrails · Group_08 · g11-g16</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>MealPlan AI  ·  g13-g17</t>
+          <t>MealPlan AI · Group_09 · g13-g17</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>MealSlot  ·  g15-g17</t>
+          <t>MealSlot · Group_10 · g15-g17</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
         <is>
-          <t>Howl2Go (G11)  ·  g17-g17</t>
+          <t>Howl2Go · Group_11 · g17-g17</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">

</xml_diff>